<commit_message>
firebase is now connected and has messages on the db, new admin panel to push new users
</commit_message>
<xml_diff>
--- a/db.xlsx
+++ b/db.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hadaritzhaki/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hadaritzhaki/Desktop/ProGmar/Hadar Pagmar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BEED18-A9D8-FE4A-B73C-7826242ECA6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A790338-86B0-454D-B133-07D7A56F8EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3660" yWindow="2760" windowWidth="27640" windowHeight="16680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5112" uniqueCount="2142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5112" uniqueCount="2143">
   <si>
     <t>תז</t>
   </si>
@@ -6450,6 +6450,9 @@
   </si>
   <si>
     <t>052-852-9418</t>
+  </si>
+  <si>
+    <t>יצחק</t>
   </si>
 </sst>
 </file>
@@ -7275,7 +7278,7 @@
         <v>18</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>19</v>
+        <v>81</v>
       </c>
       <c r="K11" s="6">
         <v>4</v>
@@ -7972,7 +7975,7 @@
         <v>26</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>19</v>
@@ -8112,7 +8115,7 @@
         <v>50</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>19</v>
@@ -8427,7 +8430,7 @@
         <v>56</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>19</v>
@@ -8462,7 +8465,7 @@
         <v>62</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J33" s="2" t="s">
         <v>19</v>
@@ -8549,7 +8552,7 @@
         <v>236</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>12</v>
+        <v>2142</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>250</v>
@@ -8567,7 +8570,7 @@
         <v>32</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J36" s="2" t="s">
         <v>19</v>
@@ -12277,7 +12280,7 @@
         <v>62</v>
       </c>
       <c r="I142" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J142" s="2" t="s">
         <v>19</v>
@@ -12347,7 +12350,7 @@
         <v>44</v>
       </c>
       <c r="I144" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J144" s="2" t="s">
         <v>19</v>
@@ -12382,7 +12385,7 @@
         <v>50</v>
       </c>
       <c r="I145" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J145" s="2" t="s">
         <v>19</v>
@@ -12522,7 +12525,7 @@
         <v>50</v>
       </c>
       <c r="I149" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J149" s="2" t="s">
         <v>19</v>
@@ -12802,7 +12805,7 @@
         <v>26</v>
       </c>
       <c r="I157" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J157" s="2" t="s">
         <v>81</v>
@@ -14132,7 +14135,7 @@
         <v>56</v>
       </c>
       <c r="I195" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J195" s="2" t="s">
         <v>19</v>
@@ -16897,7 +16900,7 @@
         <v>26</v>
       </c>
       <c r="I274" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J274" s="2" t="s">
         <v>19</v>
@@ -19277,7 +19280,7 @@
         <v>56</v>
       </c>
       <c r="I342" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J342" s="2" t="s">
         <v>81</v>
@@ -19347,7 +19350,7 @@
         <v>26</v>
       </c>
       <c r="I344" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J344" s="2" t="s">
         <v>19</v>
@@ -20467,7 +20470,7 @@
         <v>62</v>
       </c>
       <c r="I376" s="2" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="J376" s="2" t="s">
         <v>19</v>
@@ -21094,7 +21097,7 @@
         <v>80</v>
       </c>
       <c r="H394" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I394" s="2" t="s">
         <v>18</v>
@@ -21129,7 +21132,7 @@
         <v>80</v>
       </c>
       <c r="H395" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I395" s="2" t="s">
         <v>18</v>
@@ -21164,7 +21167,7 @@
         <v>80</v>
       </c>
       <c r="H396" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I396" s="2" t="s">
         <v>18</v>
@@ -21269,7 +21272,7 @@
         <v>80</v>
       </c>
       <c r="H399" s="2" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I399" s="2" t="s">
         <v>18</v>
@@ -21444,7 +21447,7 @@
         <v>80</v>
       </c>
       <c r="H404" s="2" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I404" s="2" t="s">
         <v>18</v>
@@ -21514,7 +21517,7 @@
         <v>80</v>
       </c>
       <c r="H406" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I406" s="2" t="s">
         <v>18</v>
@@ -21689,7 +21692,7 @@
         <v>80</v>
       </c>
       <c r="H411" s="2" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I411" s="2" t="s">
         <v>18</v>
@@ -21794,7 +21797,7 @@
         <v>80</v>
       </c>
       <c r="H414" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I414" s="2" t="s">
         <v>18</v>
@@ -22179,7 +22182,7 @@
         <v>80</v>
       </c>
       <c r="H425" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I425" s="2" t="s">
         <v>68</v>
@@ -22529,7 +22532,7 @@
         <v>80</v>
       </c>
       <c r="H435" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I435" s="2" t="s">
         <v>68</v>
@@ -22599,7 +22602,7 @@
         <v>80</v>
       </c>
       <c r="H437" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I437" s="2" t="s">
         <v>18</v>
@@ -22844,7 +22847,7 @@
         <v>80</v>
       </c>
       <c r="H444" s="2" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I444" s="2" t="s">
         <v>18</v>
@@ -23054,7 +23057,7 @@
         <v>80</v>
       </c>
       <c r="H450" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I450" s="2" t="s">
         <v>18</v>
@@ -23229,7 +23232,7 @@
         <v>80</v>
       </c>
       <c r="H455" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I455" s="2" t="s">
         <v>18</v>
@@ -23369,7 +23372,7 @@
         <v>80</v>
       </c>
       <c r="H459" s="2" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I459" s="2" t="s">
         <v>18</v>
@@ -23509,7 +23512,7 @@
         <v>80</v>
       </c>
       <c r="H463" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I463" s="2" t="s">
         <v>68</v>
@@ -23649,7 +23652,7 @@
         <v>80</v>
       </c>
       <c r="H467" s="2" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I467" s="2" t="s">
         <v>18</v>
@@ -23754,7 +23757,7 @@
         <v>80</v>
       </c>
       <c r="H470" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I470" s="2" t="s">
         <v>18</v>
@@ -23789,7 +23792,7 @@
         <v>80</v>
       </c>
       <c r="H471" s="2" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I471" s="2" t="s">
         <v>18</v>
@@ -23859,7 +23862,7 @@
         <v>80</v>
       </c>
       <c r="H473" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I473" s="2" t="s">
         <v>18</v>
@@ -23999,7 +24002,7 @@
         <v>80</v>
       </c>
       <c r="H477" s="2" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I477" s="2" t="s">
         <v>18</v>
@@ -24034,7 +24037,7 @@
         <v>80</v>
       </c>
       <c r="H478" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I478" s="2" t="s">
         <v>68</v>
@@ -24174,7 +24177,7 @@
         <v>80</v>
       </c>
       <c r="H482" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I482" s="2" t="s">
         <v>68</v>
@@ -24244,7 +24247,7 @@
         <v>80</v>
       </c>
       <c r="H484" s="2" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I484" s="2" t="s">
         <v>18</v>
@@ -24279,7 +24282,7 @@
         <v>80</v>
       </c>
       <c r="H485" s="2" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I485" s="2" t="s">
         <v>18</v>
@@ -24454,7 +24457,7 @@
         <v>80</v>
       </c>
       <c r="H490" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I490" s="2" t="s">
         <v>18</v>
@@ -24559,7 +24562,7 @@
         <v>80</v>
       </c>
       <c r="H493" s="2" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I493" s="2" t="s">
         <v>18</v>
@@ -24699,7 +24702,7 @@
         <v>80</v>
       </c>
       <c r="H497" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I497" s="2" t="s">
         <v>18</v>
@@ -24734,7 +24737,7 @@
         <v>80</v>
       </c>
       <c r="H498" s="2" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="I498" s="2" t="s">
         <v>18</v>

</xml_diff>